<commit_message>
Remove the 45-minute interview limit from the instrument's text and notes
No questions changed. The time cap was not verifiable before fieldwork, so it is no longer
stated as a design constraint. Interview length is still recorded from the tablet's timestamps.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Question_register.xlsx
+++ b/Question_register.xlsx
@@ -8318,7 +8318,7 @@
       <c r="I172" s="2" t="inlineStr"/>
       <c r="J172" s="2" t="inlineStr">
         <is>
-          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, left out to stay inside the 45-minute limit. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking; a day-count also takes about as long to answer as a yes/no in practice, so little interview time is saved by simplifying it.</t>
+          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, which is not included in this instrument. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking.</t>
         </is>
       </c>
     </row>
@@ -8360,7 +8360,7 @@
       <c r="I173" s="2" t="inlineStr"/>
       <c r="J173" s="2" t="inlineStr">
         <is>
-          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, left out to stay inside the 45-minute limit. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking; a day-count also takes about as long to answer as a yes/no in practice, so little interview time is saved by simplifying it.</t>
+          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, which is not included in this instrument. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking.</t>
         </is>
       </c>
     </row>
@@ -8402,7 +8402,7 @@
       <c r="I174" s="2" t="inlineStr"/>
       <c r="J174" s="2" t="inlineStr">
         <is>
-          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, left out to stay inside the 45-minute limit. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking; a day-count also takes about as long to answer as a yes/no in practice, so little interview time is saved by simplifying it.</t>
+          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, which is not included in this instrument. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking.</t>
         </is>
       </c>
     </row>
@@ -8444,7 +8444,7 @@
       <c r="I175" s="2" t="inlineStr"/>
       <c r="J175" s="2" t="inlineStr">
         <is>
-          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, left out to stay inside the 45-minute limit. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking; a day-count also takes about as long to answer as a yes/no in practice, so little interview time is saved by simplifying it.</t>
+          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, which is not included in this instrument. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking.</t>
         </is>
       </c>
     </row>
@@ -8486,7 +8486,7 @@
       <c r="I176" s="2" t="inlineStr"/>
       <c r="J176" s="2" t="inlineStr">
         <is>
-          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, left out to stay inside the 45-minute limit. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking; a day-count also takes about as long to answer as a yes/no in practice, so little interview time is saved by simplifying it.</t>
+          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, which is not included in this instrument. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking.</t>
         </is>
       </c>
     </row>
@@ -8528,7 +8528,7 @@
       <c r="I177" s="2" t="inlineStr"/>
       <c r="J177" s="2" t="inlineStr">
         <is>
-          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, left out to stay inside the 45-minute limit. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking; a day-count also takes about as long to answer as a yes/no in practice, so little interview time is saved by simplifying it.</t>
+          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, which is not included in this instrument. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking.</t>
         </is>
       </c>
     </row>
@@ -8570,7 +8570,7 @@
       <c r="I178" s="2" t="inlineStr"/>
       <c r="J178" s="2" t="inlineStr">
         <is>
-          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, left out to stay inside the 45-minute limit. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking; a day-count also takes about as long to answer as a yes/no in practice, so little interview time is saved by simplifying it.</t>
+          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, which is not included in this instrument. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking.</t>
         </is>
       </c>
     </row>
@@ -8612,7 +8612,7 @@
       <c r="I179" s="2" t="inlineStr"/>
       <c r="J179" s="2" t="inlineStr">
         <is>
-          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, left out to stay inside the 45-minute limit. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking; a day-count also takes about as long to answer as a yes/no in practice, so little interview time is saved by simplifying it.</t>
+          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, which is not included in this instrument. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking.</t>
         </is>
       </c>
     </row>
@@ -8654,7 +8654,7 @@
       <c r="I180" s="2" t="inlineStr"/>
       <c r="J180" s="2" t="inlineStr">
         <is>
-          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, left out to stay inside the 45-minute limit. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking; a day-count also takes about as long to answer as a yes/no in practice, so little interview time is saved by simplifying it.</t>
+          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, which is not included in this instrument. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking.</t>
         </is>
       </c>
     </row>
@@ -8696,7 +8696,7 @@
       <c r="I181" s="2" t="inlineStr"/>
       <c r="J181" s="2" t="inlineStr">
         <is>
-          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, left out to stay inside the 45-minute limit. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking; a day-count also takes about as long to answer as a yes/no in practice, so little interview time is saved by simplifying it.</t>
+          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, which is not included in this instrument. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking.</t>
         </is>
       </c>
     </row>
@@ -15583,7 +15583,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, left out to stay inside the 45-minute limit. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking; a day-count also takes about as long to answer as a yes/no in practice, so little interview time is saved by simplifying it.</t>
+          <t>VASyR 2025 (exact item wording); WFP rCSI; The reduced Coping Strategy Index (rCSI): five food-coping questions, standard WFP weights (1, 2, 1, 1, 3) applied when the index is built. The Kedarnath instrument otherwise has no food-security module, which is a gap for a poverty-vulnerability survey; these five short questions close it at low cost instead of a full dietary-diversity module, which is not included in this instrument. Kept as day-counts (0-7), not collapsed to yes/no: this is the standard, validated WFP/FAO specification (frequency x severity), and no comparably-standard binary version was found on checking.</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">

</xml_diff>